<commit_message>
Update 18 Nov 2025: Orientasi print dan PDF.
</commit_message>
<xml_diff>
--- a/file 1.xlsx
+++ b/file 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NITIB\batch_print\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169950F2-5A1C-4B9B-AF40-438DF42C0572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17C5FF9-4883-438F-8026-3225B2FCFC8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{0EC7FDE0-C78D-4BC0-A9D0-A57FC56FAB99}"/>
   </bookViews>
@@ -1380,24 +1380,24 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1407,6 +1407,75 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1443,12 +1512,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1470,15 +1533,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1492,60 +1546,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3213,56 +3213,56 @@
     </row>
     <row r="4" spans="1:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="1:12" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="97" t="s">
+      <c r="A5" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="93"/>
-      <c r="C5" s="93" t="s">
+      <c r="B5" s="94"/>
+      <c r="C5" s="94" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93" t="s">
+      <c r="D5" s="94"/>
+      <c r="E5" s="94" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93" t="s">
+      <c r="F5" s="94"/>
+      <c r="G5" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93" t="s">
+      <c r="H5" s="94"/>
+      <c r="I5" s="94" t="s">
         <v>40</v>
       </c>
-      <c r="J5" s="93"/>
-      <c r="K5" s="93" t="s">
+      <c r="J5" s="94"/>
+      <c r="K5" s="94" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="94"/>
+      <c r="L5" s="97"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="98">
+      <c r="A6" s="95">
         <v>1</v>
       </c>
-      <c r="B6" s="95"/>
-      <c r="C6" s="95">
+      <c r="B6" s="96"/>
+      <c r="C6" s="96">
         <v>2</v>
       </c>
-      <c r="D6" s="95"/>
-      <c r="E6" s="95">
+      <c r="D6" s="96"/>
+      <c r="E6" s="96">
         <v>3</v>
       </c>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95">
+      <c r="F6" s="96"/>
+      <c r="G6" s="96">
         <v>4</v>
       </c>
-      <c r="H6" s="95"/>
-      <c r="I6" s="95">
+      <c r="H6" s="96"/>
+      <c r="I6" s="96">
         <v>5</v>
       </c>
-      <c r="J6" s="95"/>
-      <c r="K6" s="95">
+      <c r="J6" s="96"/>
+      <c r="K6" s="96">
         <v>6</v>
       </c>
-      <c r="L6" s="96"/>
+      <c r="L6" s="98"/>
     </row>
     <row r="7" spans="1:12" s="10" customFormat="1" ht="101.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="77" t="s">
@@ -3421,22 +3421,22 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="K6:L6"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="K6:L6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.69291338582677164" right="0.69291338582677164" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="72" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3743,54 +3743,54 @@
     <row r="1" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="28"/>
       <c r="B1" s="29"/>
-      <c r="C1" s="107" t="s">
+      <c r="C1" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="108"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="113"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="136"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="30"/>
       <c r="B2" s="31"/>
-      <c r="C2" s="107" t="s">
+      <c r="C2" s="130" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="108"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="119"/>
+      <c r="D2" s="131"/>
+      <c r="E2" s="139"/>
+      <c r="F2" s="140"/>
     </row>
     <row r="3" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11"/>
       <c r="B3" s="31"/>
-      <c r="C3" s="107" t="s">
+      <c r="C3" s="130" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="108"/>
-      <c r="E3" s="116"/>
-      <c r="F3" s="117"/>
+      <c r="D3" s="131"/>
+      <c r="E3" s="137"/>
+      <c r="F3" s="138"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11"/>
       <c r="B4" s="32"/>
-      <c r="C4" s="107" t="s">
+      <c r="C4" s="130" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="108"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="130"/>
+      <c r="D4" s="131"/>
+      <c r="E4" s="147"/>
+      <c r="F4" s="148"/>
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
       <c r="B5" s="32"/>
-      <c r="C5" s="109" t="s">
+      <c r="C5" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="110"/>
-      <c r="E5" s="102" t="s">
+      <c r="D5" s="133"/>
+      <c r="E5" s="125" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="103"/>
+      <c r="F5" s="126"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
@@ -3799,10 +3799,10 @@
       <c r="B6" s="32"/>
       <c r="C6" s="71"/>
       <c r="D6" s="72"/>
-      <c r="E6" s="114" t="s">
+      <c r="E6" s="102" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="115"/>
+      <c r="F6" s="103"/>
     </row>
     <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
@@ -3825,51 +3825,51 @@
       <c r="B9" s="32"/>
       <c r="C9" s="71"/>
       <c r="D9" s="72"/>
-      <c r="E9" s="114" t="s">
+      <c r="E9" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="F9" s="115"/>
+      <c r="F9" s="103"/>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="30"/>
       <c r="B10" s="32"/>
       <c r="C10" s="71"/>
       <c r="D10" s="72"/>
-      <c r="E10" s="114" t="s">
+      <c r="E10" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="115"/>
+      <c r="F10" s="103"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="33"/>
       <c r="B11" s="34"/>
       <c r="C11" s="35"/>
       <c r="D11" s="36"/>
-      <c r="E11" s="144" t="s">
+      <c r="E11" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="F11" s="145"/>
+      <c r="F11" s="105"/>
     </row>
     <row r="12" spans="1:6" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="37" t="s">
         <v>98</v>
       </c>
       <c r="B12" s="38"/>
-      <c r="C12" s="111" t="s">
+      <c r="C12" s="134" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="112"/>
-      <c r="E12" s="131" t="s">
+      <c r="D12" s="135"/>
+      <c r="E12" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="F12" s="132"/>
+      <c r="F12" s="113"/>
     </row>
     <row r="13" spans="1:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="66"/>
       <c r="B13" s="67"/>
-      <c r="C13" s="143"/>
-      <c r="D13" s="143"/>
-      <c r="E13" s="143"/>
+      <c r="C13" s="124"/>
+      <c r="D13" s="124"/>
+      <c r="E13" s="124"/>
       <c r="F13" s="68"/>
     </row>
     <row r="14" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3877,97 +3877,97 @@
         <v>9</v>
       </c>
       <c r="B14" s="54"/>
-      <c r="C14" s="146" t="s">
+      <c r="C14" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="147"/>
-      <c r="E14" s="147"/>
-      <c r="F14" s="148"/>
+      <c r="D14" s="110"/>
+      <c r="E14" s="110"/>
+      <c r="F14" s="111"/>
     </row>
     <row r="15" spans="1:6" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="120" t="s">
+      <c r="C15" s="141" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="121"/>
-      <c r="E15" s="121"/>
-      <c r="F15" s="122"/>
+      <c r="D15" s="142"/>
+      <c r="E15" s="142"/>
+      <c r="F15" s="143"/>
     </row>
     <row r="16" spans="1:6" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="123" t="s">
+      <c r="C16" s="106" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="124"/>
-      <c r="E16" s="124"/>
-      <c r="F16" s="125"/>
+      <c r="D16" s="107"/>
+      <c r="E16" s="107"/>
+      <c r="F16" s="108"/>
     </row>
     <row r="17" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="80" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="123" t="s">
+      <c r="C17" s="106" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="124"/>
-      <c r="E17" s="124"/>
-      <c r="F17" s="125"/>
+      <c r="D17" s="107"/>
+      <c r="E17" s="107"/>
+      <c r="F17" s="108"/>
     </row>
     <row r="18" spans="1:6" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="51"/>
-      <c r="C18" s="123"/>
-      <c r="D18" s="124"/>
-      <c r="E18" s="124"/>
-      <c r="F18" s="125"/>
+      <c r="C18" s="106"/>
+      <c r="D18" s="107"/>
+      <c r="E18" s="107"/>
+      <c r="F18" s="108"/>
     </row>
     <row r="19" spans="1:6" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="48"/>
-      <c r="C19" s="123"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="125"/>
+      <c r="C19" s="106"/>
+      <c r="D19" s="107"/>
+      <c r="E19" s="107"/>
+      <c r="F19" s="108"/>
     </row>
     <row r="20" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="49" t="s">
         <v>11</v>
       </c>
       <c r="B20" s="55"/>
-      <c r="C20" s="134" t="s">
+      <c r="C20" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="135"/>
-      <c r="E20" s="135"/>
-      <c r="F20" s="136"/>
+      <c r="D20" s="116"/>
+      <c r="E20" s="116"/>
+      <c r="F20" s="117"/>
     </row>
     <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="133"/>
-      <c r="C21" s="137" t="s">
+      <c r="B21" s="114"/>
+      <c r="C21" s="118" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="138"/>
-      <c r="E21" s="138"/>
-      <c r="F21" s="139"/>
+      <c r="D21" s="119"/>
+      <c r="E21" s="119"/>
+      <c r="F21" s="120"/>
     </row>
     <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="133"/>
-      <c r="C22" s="140"/>
-      <c r="D22" s="141"/>
-      <c r="E22" s="141"/>
-      <c r="F22" s="142"/>
+      <c r="B22" s="114"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="122"/>
+      <c r="E22" s="122"/>
+      <c r="F22" s="123"/>
     </row>
     <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="51"/>
-      <c r="B23" s="133"/>
+      <c r="B23" s="114"/>
       <c r="C23" s="81" t="s">
         <v>59</v>
       </c>
@@ -3977,7 +3977,7 @@
     </row>
     <row r="24" spans="1:6" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="52"/>
-      <c r="B24" s="133"/>
+      <c r="B24" s="114"/>
       <c r="C24" s="83" t="s">
         <v>60</v>
       </c>
@@ -3990,39 +3990,27 @@
         <v>13</v>
       </c>
       <c r="B25" s="55"/>
-      <c r="C25" s="126" t="s">
+      <c r="C25" s="144" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="127"/>
-      <c r="E25" s="127"/>
-      <c r="F25" s="128"/>
+      <c r="D25" s="145"/>
+      <c r="E25" s="145"/>
+      <c r="F25" s="146"/>
     </row>
     <row r="26" spans="1:6" ht="66.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="39" t="s">
         <v>67</v>
       </c>
       <c r="B26" s="40"/>
-      <c r="C26" s="104" t="s">
+      <c r="C26" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="D26" s="105"/>
-      <c r="E26" s="105"/>
-      <c r="F26" s="106"/>
+      <c r="D26" s="128"/>
+      <c r="E26" s="128"/>
+      <c r="F26" s="129"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B21:B24"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F22"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="C18:F18"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="C26:F26"/>
     <mergeCell ref="C1:D1"/>
@@ -4039,10 +4027,22 @@
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="C25:F25"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F22"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="E12:F12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.69291338582677164" right="0.69291338582677164" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="61" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="92" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>

</xml_diff>